<commit_message>
Add alternative sales and spend calculation
Co-authored-by: mail135797 <mail135797@gmail.com>
</commit_message>
<xml_diff>
--- a/second_data.xlsx
+++ b/second_data.xlsx
@@ -8,13 +8,14 @@
   </bookViews>
   <sheets>
     <sheet name="second_data" sheetId="1" r:id="rId1"/>
+    <sheet name="second_data_alt" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>항목</t>
   </si>
@@ -38,6 +39,21 @@
   </si>
   <si>
     <t>타사 상품(ASIN) 타게팅 경유 매상 총합</t>
+  </si>
+  <si>
+    <t>before_spend_alloc</t>
+  </si>
+  <si>
+    <t>after_spend_alloc</t>
+  </si>
+  <si>
+    <t>자사(광고된 SKU) 매상 총합</t>
+  </si>
+  <si>
+    <t>기타(그 외 SKU) 매상 총합</t>
+  </si>
+  <si>
+    <t>총 매상(검색어 리포트)</t>
   </si>
 </sst>
 </file>
@@ -402,7 +418,7 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
+    <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="5" width="18.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -477,4 +493,86 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="5" width="20.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1977364</v>
+      </c>
+      <c r="C2" s="1">
+        <v>954975</v>
+      </c>
+      <c r="D2" s="1">
+        <v>331846.7271309997</v>
+      </c>
+      <c r="E2" s="1">
+        <v>120874.4352571916</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2362320</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1698029</v>
+      </c>
+      <c r="D3" s="1">
+        <v>324604.1728690004</v>
+      </c>
+      <c r="E3" s="1">
+        <v>152486.6347428084</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1">
+        <v>4339684</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2653004</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1370884.87</v>
+      </c>
+      <c r="E4" s="1">
+        <v>1099928.28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>